<commit_message>
add and start analyze sub-hypothesis
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A9A942-0C36-4029-ADA5-C50C4F2A7353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951FB732-35CB-4829-A4A4-6E8CF01563CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
@@ -588,7 +588,7 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
@@ -614,7 +614,7 @@
       <c r="B5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J5" t="s">
@@ -657,6 +657,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -667,16 +676,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -925,15 +933,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -944,15 +952,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -969,16 +981,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add to theory - BS reform process, SH details
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951FB732-35CB-4829-A4A4-6E8CF01563CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8846E87-FBDB-4873-B6BF-EB6CBFDD4C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
   <si>
     <t>KW38</t>
   </si>
@@ -66,9 +66,6 @@
     <t>Datasourcing</t>
   </si>
   <si>
-    <t>before KW38</t>
-  </si>
-  <si>
     <t>Datacleaning finish</t>
   </si>
   <si>
@@ -108,9 +105,6 @@
     <t>Timeplan Thesis</t>
   </si>
   <si>
-    <t>Tasks</t>
-  </si>
-  <si>
     <t>finish Analysis broadly</t>
   </si>
   <si>
@@ -136,6 +130,24 @@
   </si>
   <si>
     <t>integrate canton specifications</t>
+  </si>
+  <si>
+    <t>Continue analysis</t>
+  </si>
+  <si>
+    <t>KW 34-37</t>
+  </si>
+  <si>
+    <t>before KW  34</t>
+  </si>
+  <si>
+    <t>Datacollection</t>
+  </si>
+  <si>
+    <t>Preparation</t>
+  </si>
+  <si>
+    <t>Structure Datacleaning</t>
   </si>
 </sst>
 </file>
@@ -497,7 +509,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="23" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -512,8 +524,11 @@
       <c r="L1" s="4"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>0</v>
@@ -543,102 +558,111 @@
         <v>8</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>24</v>
+      <c r="A3" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" t="s">
-        <v>27</v>
-      </c>
-      <c r="K3" t="s">
-        <v>16</v>
-      </c>
       <c r="L3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
       </c>
       <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
         <v>26</v>
       </c>
-      <c r="F4" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" t="s">
-        <v>28</v>
-      </c>
       <c r="K4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -657,15 +681,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -676,15 +691,16 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -933,15 +949,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -952,19 +968,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -981,4 +993,16 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add theory: expected effects of transition, adjust timeplan
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8846E87-FBDB-4873-B6BF-EB6CBFDD4C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1CA5CB0-4315-402D-A621-7C2A3889E17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
   <si>
     <t>KW38</t>
   </si>
@@ -93,9 +93,6 @@
     <t>AI declaration</t>
   </si>
   <si>
-    <t>continue Analysis (deeper)</t>
-  </si>
-  <si>
     <t>Datacleaning</t>
   </si>
   <si>
@@ -108,9 +105,6 @@
     <t>finish Analysis broadly</t>
   </si>
   <si>
-    <t>finish Theory /Lit.Review</t>
-  </si>
-  <si>
     <t>Check Thesis</t>
   </si>
   <si>
@@ -123,9 +117,6 @@
     <t>Conclusion</t>
   </si>
   <si>
-    <t>open</t>
-  </si>
-  <si>
     <t>finish analysis add final touch</t>
   </si>
   <si>
@@ -148,6 +139,18 @@
   </si>
   <si>
     <t>Structure Datacleaning</t>
+  </si>
+  <si>
+    <t>continue analysis deeper</t>
+  </si>
+  <si>
+    <t>continue Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> broadly finish Theory /Lit.Review</t>
+  </si>
+  <si>
+    <t>finish theory / lit review</t>
   </si>
 </sst>
 </file>
@@ -211,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -221,6 +224,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -509,7 +513,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="23" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -525,10 +529,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>0</v>
@@ -563,10 +567,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>10</v>
@@ -575,22 +579,22 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
         <v>23</v>
-      </c>
-      <c r="G3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>25</v>
       </c>
       <c r="K3" t="s">
         <v>15</v>
@@ -601,7 +605,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
@@ -610,19 +614,19 @@
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" t="s">
         <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4" t="s">
-        <v>26</v>
       </c>
       <c r="K4" t="s">
         <v>15</v>
@@ -633,13 +637,16 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J5" t="s">
         <v>17</v>
@@ -681,6 +688,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -691,16 +707,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -949,15 +964,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -968,15 +983,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -993,16 +1012,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add theory: lit.review extend part
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -214,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -224,7 +224,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,7 +580,7 @@
       <c r="E3" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" t="s">
         <v>35</v>
       </c>
       <c r="G3" t="s">
@@ -645,7 +644,7 @@
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" t="s">
         <v>38</v>
       </c>
       <c r="J5" t="s">
@@ -688,15 +687,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -707,15 +697,16 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -964,15 +955,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -983,19 +974,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1012,4 +999,16 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
write Research Design & Counterfactual strategy part
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1CA5CB0-4315-402D-A621-7C2A3889E17C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B75417-5FA5-4EEA-A2F0-037CA7263EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="42">
   <si>
     <t>KW38</t>
   </si>
@@ -151,6 +151,15 @@
   </si>
   <si>
     <t>finish theory / lit review</t>
+  </si>
+  <si>
+    <t>fully achieved</t>
+  </si>
+  <si>
+    <t>partly achieved</t>
+  </si>
+  <si>
+    <t>not achieved</t>
   </si>
 </sst>
 </file>
@@ -188,7 +197,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,6 +207,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -214,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -224,6 +245,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -504,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D97C9A4-50BE-496C-B8D0-1CBB038FD110}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="12" width="20.58203125" customWidth="1"/>
@@ -574,7 +597,7 @@
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E3" t="s">
@@ -612,7 +635,7 @@
       <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="5" t="s">
         <v>29</v>
       </c>
       <c r="E4" t="s">
@@ -669,6 +692,21 @@
       </c>
       <c r="L6" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -687,6 +725,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -697,16 +744,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -955,15 +1001,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -974,15 +1020,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -999,16 +1049,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
finish data sources part
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B75417-5FA5-4EEA-A2F0-037CA7263EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3C6CCB-D0F5-4FF7-9E69-9167F1ACFDC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -120,9 +120,6 @@
     <t>finish analysis add final touch</t>
   </si>
   <si>
-    <t>integrate canton specifications</t>
-  </si>
-  <si>
     <t>Continue analysis</t>
   </si>
   <si>
@@ -160,6 +157,9 @@
   </si>
   <si>
     <t>not achieved</t>
+  </si>
+  <si>
+    <t>integrate canton specifications in results</t>
   </si>
 </sst>
 </file>
@@ -197,7 +197,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -222,6 +222,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -235,18 +241,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,27 +541,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>0</v>
@@ -589,7 +596,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>20</v>
@@ -600,11 +607,11 @@
       <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
-        <v>36</v>
+      <c r="E3" s="7" t="s">
+        <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G3" t="s">
         <v>22</v>
@@ -627,7 +634,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
@@ -635,14 +642,14 @@
       <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
+      <c r="D4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="I4" t="s">
         <v>26</v>
@@ -659,7 +666,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>19</v>
@@ -667,8 +674,8 @@
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F5" t="s">
-        <v>38</v>
+      <c r="F5" s="7" t="s">
+        <v>37</v>
       </c>
       <c r="J5" t="s">
         <v>17</v>
@@ -696,17 +703,17 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>40</v>
+      <c r="A11" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>41</v>
+      <c r="A12" s="4" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -725,15 +732,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -744,15 +742,16 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -1001,15 +1000,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1020,19 +1019,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1049,4 +1044,16 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
revise first parts of thesis
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3C6CCB-D0F5-4FF7-9E69-9167F1ACFDC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -247,13 +247,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,20 +541,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -607,7 +607,7 @@
       <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F3" t="s">
@@ -645,7 +645,7 @@
       <c r="D4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>36</v>
       </c>
       <c r="F4" t="s">
@@ -674,7 +674,7 @@
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>37</v>
       </c>
       <c r="J5" t="s">
@@ -732,6 +732,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -742,16 +751,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -1000,15 +1008,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1019,15 +1027,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1044,16 +1056,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
start summing analysis eq2, update timeplan
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3C6CCB-D0F5-4FF7-9E69-9167F1ACFDC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE36C92-FE2B-45FD-9C31-0509BA35DC1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
@@ -197,7 +197,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -228,6 +228,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -241,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -254,6 +260,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,7 +617,7 @@
       <c r="E3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="8" t="s">
         <v>34</v>
       </c>
       <c r="G3" t="s">
@@ -648,7 +655,7 @@
       <c r="E4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="8" t="s">
         <v>41</v>
       </c>
       <c r="I4" t="s">
@@ -732,15 +739,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -751,15 +749,16 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -1008,15 +1007,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1027,19 +1026,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1056,4 +1051,16 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
precise Aargau case in EQ3, continue analysis EQ4
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE36C92-FE2B-45FD-9C31-0509BA35DC1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF096D3F-010C-4E32-88CC-935320B9F50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
   <si>
     <t>KW38</t>
   </si>
@@ -160,6 +160,9 @@
   </si>
   <si>
     <t>integrate canton specifications in results</t>
+  </si>
+  <si>
+    <t>clean code add notations</t>
   </si>
 </sst>
 </file>
@@ -254,13 +257,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,20 +551,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -617,7 +620,7 @@
       <c r="E3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="6" t="s">
         <v>34</v>
       </c>
       <c r="G3" t="s">
@@ -655,8 +658,11 @@
       <c r="E4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>41</v>
+      </c>
+      <c r="H4" t="s">
+        <v>42</v>
       </c>
       <c r="I4" t="s">
         <v>26</v>
@@ -683,6 +689,9 @@
       </c>
       <c r="F5" s="5" t="s">
         <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>23</v>
       </c>
       <c r="J5" t="s">
         <v>17</v>
@@ -739,6 +748,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -749,16 +767,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -1007,15 +1024,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1026,15 +1043,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1051,16 +1072,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
extend H1 results, based on new figure, expand Appendix with supplemenatary graph, explanation etc
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF096D3F-010C-4E32-88CC-935320B9F50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4078B8B-0F9D-4773-B895-1BF738AAA843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -623,7 +623,7 @@
       <c r="F3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="5" t="s">
         <v>22</v>
       </c>
       <c r="H3" t="s">
@@ -748,15 +748,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -767,15 +758,16 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -1024,15 +1016,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1043,19 +1035,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1072,4 +1060,16 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
improving visualizations according to measures
</commit_message>
<xml_diff>
--- a/formalities/timeplan_broad.xlsx
+++ b/formalities/timeplan_broad.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moritz\Desktop\HSG\BA\BA_Thesis\formalities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4078B8B-0F9D-4773-B895-1BF738AAA843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7753FD0C-B20A-43B3-B5D6-0CC52E3BB496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A6D6FD58-BABA-4C76-B2FD-B993785552B7}"/>
   </bookViews>
@@ -748,6 +748,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="07c8a24f-8b40-44ca-950f-ae5db2c4fa23">
@@ -758,16 +767,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010034C2EED3AEDAB24AB48AF05A7A255DF4" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="274d9017fadbcc8b67afbe4b22a55600">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="07c8a24f-8b40-44ca-950f-ae5db2c4fa23" xmlns:ns3="71d337dc-809a-4269-a690-d6cd31b4acd0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0b58614a3de855f8a451fa93eb2e43b4" ns2:_="" ns3:_="">
     <xsd:import namespace="07c8a24f-8b40-44ca-950f-ae5db2c4fa23"/>
@@ -1016,15 +1024,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"UNISG Excel hoch","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0002BB93-0A85-478E-910B-252B9B8A5C15}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1035,15 +1043,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC0B089E-410A-4C91-B0A8-BAA2927F78EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
+  <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F268B634-479A-4DE9-9C23-26EB34AB525F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1060,16 +1072,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62C84976-48B0-49F1-88C9-1A6F278B1636}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4F7B3D-00BA-4EC3-B5E5-E2B2297DE47E}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
 </file>
</xml_diff>